<commit_message>
fix: complete all 22 regions to official district counts
- 台中市 28→29區（補大安區）
- 台南市 16→37區（補21區）
- 高雄市 16→38區（補22區）
- 屏東縣 16→33鄉鎮市（補17個）

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/excel/04-taichung.xlsx
+++ b/data/excel/04-taichung.xlsx
@@ -4510,7 +4510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D113"/>
+  <dimension ref="A1:D117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5088,12 +5088,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>豐原區</t>
+          <t>太平區</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>豐原廟東夜市</t>
+          <t>太平市區</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -5105,12 +5105,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>豐原區</t>
+          <t>太平區</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>豐原市區</t>
+          <t>中山路</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -5122,12 +5122,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>豐原區</t>
+          <t>太平區</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>中山路</t>
+          <t>長億路</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -5139,12 +5139,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>豐原區</t>
+          <t>太平區</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>豐勢路</t>
+          <t>新興路</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -5224,12 +5224,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>太平區</t>
+          <t>霧峰區</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>太平市區</t>
+          <t>霧峰市區</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -5241,12 +5241,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>太平區</t>
+          <t>霧峰區</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>中山路</t>
+          <t>光復新村</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -5258,12 +5258,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>太平區</t>
+          <t>霧峰區</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>長億路</t>
+          <t>亞洲大學周邊</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -5275,12 +5275,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>太平區</t>
+          <t>霧峰區</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>新興路</t>
+          <t>萬豐路</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -5292,12 +5292,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>清水區</t>
+          <t>烏日區</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>清水市區</t>
+          <t>高鐵台中站特區</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -5309,12 +5309,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>清水區</t>
+          <t>烏日區</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>清水老街</t>
+          <t>烏日市區</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -5326,7 +5326,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>清水區</t>
+          <t>烏日區</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -5343,12 +5343,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>清水區</t>
+          <t>烏日區</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>清水港路</t>
+          <t>成功路</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -5360,12 +5360,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>梧棲區</t>
+          <t>豐原區</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>梧棲漁港</t>
+          <t>豐原廟東夜市</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -5377,12 +5377,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>梧棲區</t>
+          <t>豐原區</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>梧棲市區</t>
+          <t>豐原市區</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -5394,7 +5394,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>梧棲區</t>
+          <t>豐原區</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -5411,12 +5411,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>梧棲區</t>
+          <t>豐原區</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>文化路</t>
+          <t>豐勢路</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -5428,12 +5428,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>沙鹿區</t>
+          <t>后里區</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>沙鹿市區</t>
+          <t>后里市區</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -5445,12 +5445,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>沙鹿區</t>
+          <t>后里區</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>中山路</t>
+          <t>麗寶樂園</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -5462,12 +5462,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>沙鹿區</t>
+          <t>后里區</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>鎮政路</t>
+          <t>月眉</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -5479,12 +5479,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>沙鹿區</t>
+          <t>后里區</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>竹林路</t>
+          <t>中山路</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -5496,12 +5496,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>龍井區</t>
+          <t>石岡區</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>龍井市區</t>
+          <t>石岡市區</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -5513,7 +5513,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>龍井區</t>
+          <t>石岡區</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -5530,12 +5530,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>龍井區</t>
+          <t>石岡區</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>台中港周邊</t>
+          <t>食水嵙</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -5547,12 +5547,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>龍井區</t>
+          <t>石岡區</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>龍井社口</t>
+          <t>三叉坑</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -5564,12 +5564,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>大肚區</t>
+          <t>東勢區</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>大肚市區</t>
+          <t>東勢市區</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -5581,12 +5581,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>大肚區</t>
+          <t>東勢區</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>中山路</t>
+          <t>東勢水果市場</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -5598,12 +5598,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>大肚區</t>
+          <t>東勢區</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>永和路</t>
+          <t>中山路</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -5615,12 +5615,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>大肚區</t>
+          <t>東勢區</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>大肚山</t>
+          <t>本街</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -5632,12 +5632,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>烏日區</t>
+          <t>和平區</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>高鐵台中站特區</t>
+          <t>梨山</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -5649,12 +5649,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>烏日區</t>
+          <t>和平區</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>烏日市區</t>
+          <t>武陵農場</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -5666,12 +5666,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>烏日區</t>
+          <t>和平區</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>中山路</t>
+          <t>谷關溫泉</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -5683,12 +5683,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>烏日區</t>
+          <t>和平區</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>成功路</t>
+          <t>環山部落</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -5700,12 +5700,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>霧峰區</t>
+          <t>新社區</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>霧峰市區</t>
+          <t>新社市區</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -5717,12 +5717,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>霧峰區</t>
+          <t>新社區</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>光復新村</t>
+          <t>新社花海</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -5734,12 +5734,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>霧峰區</t>
+          <t>新社區</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>亞洲大學周邊</t>
+          <t>中山路</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -5751,12 +5751,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>霧峰區</t>
+          <t>新社區</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>萬豐路</t>
+          <t>古堡花園</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -5768,12 +5768,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>大甲區</t>
+          <t>潭子區</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>大甲市區</t>
+          <t>潭子市區</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -5785,12 +5785,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>大甲區</t>
+          <t>潭子區</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>大甲媽祖</t>
+          <t>潭子火車站</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -5802,7 +5802,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>大甲區</t>
+          <t>潭子區</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -5819,12 +5819,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>大甲區</t>
+          <t>潭子區</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>蔣公路</t>
+          <t>雅潭路</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -5836,12 +5836,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>外埔區</t>
+          <t>大雅區</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>外埔市區</t>
+          <t>大雅市區</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -5853,7 +5853,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>外埔區</t>
+          <t>大雅區</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -5870,12 +5870,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>外埔區</t>
+          <t>大雅區</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>大甲溪</t>
+          <t>中清路</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -5887,12 +5887,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>外埔區</t>
+          <t>大雅區</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>水美溫泉</t>
+          <t>小麥文化節</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -5904,12 +5904,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>后里區</t>
+          <t>神岡區</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>后里市區</t>
+          <t>神岡市區</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -5921,12 +5921,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>后里區</t>
+          <t>神岡區</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>麗寶樂園</t>
+          <t>中山路</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -5938,12 +5938,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>后里區</t>
+          <t>神岡區</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>月眉</t>
+          <t>三民路</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -5955,12 +5955,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>后里區</t>
+          <t>神岡區</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>中山路</t>
+          <t>豐洲科技</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -5972,12 +5972,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>神岡區</t>
+          <t>大肚區</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>神岡市區</t>
+          <t>大肚市區</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -5989,7 +5989,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>神岡區</t>
+          <t>大肚區</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -6006,12 +6006,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>神岡區</t>
+          <t>大肚區</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>三民路</t>
+          <t>永和路</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -6023,12 +6023,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>神岡區</t>
+          <t>大肚區</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>豐洲科技</t>
+          <t>大肚山</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -6040,12 +6040,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>大雅區</t>
+          <t>沙鹿區</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>大雅市區</t>
+          <t>沙鹿市區</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -6057,7 +6057,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>大雅區</t>
+          <t>沙鹿區</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -6074,12 +6074,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>大雅區</t>
+          <t>沙鹿區</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>中清路</t>
+          <t>鎮政路</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -6091,12 +6091,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>大雅區</t>
+          <t>沙鹿區</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>小麥文化節</t>
+          <t>竹林路</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -6108,12 +6108,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>潭子區</t>
+          <t>龍井區</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>潭子市區</t>
+          <t>龍井市區</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -6125,12 +6125,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>潭子區</t>
+          <t>龍井區</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>潭子火車站</t>
+          <t>中山路</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -6142,12 +6142,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>潭子區</t>
+          <t>龍井區</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>中山路</t>
+          <t>台中港周邊</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -6159,12 +6159,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>潭子區</t>
+          <t>龍井區</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>雅潭路</t>
+          <t>龍井社口</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -6176,12 +6176,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>新社區</t>
+          <t>梧棲區</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>新社市區</t>
+          <t>梧棲漁港</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -6193,12 +6193,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>新社區</t>
+          <t>梧棲區</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>新社花海</t>
+          <t>梧棲市區</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -6210,7 +6210,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>新社區</t>
+          <t>梧棲區</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -6227,12 +6227,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>新社區</t>
+          <t>梧棲區</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>古堡花園</t>
+          <t>文化路</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -6244,12 +6244,12 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>東勢區</t>
+          <t>清水區</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>東勢市區</t>
+          <t>清水市區</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -6261,12 +6261,12 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>東勢區</t>
+          <t>清水區</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>東勢水果市場</t>
+          <t>清水老街</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -6278,7 +6278,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>東勢區</t>
+          <t>清水區</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -6295,12 +6295,12 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>東勢區</t>
+          <t>清水區</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>本街</t>
+          <t>清水港路</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -6312,12 +6312,12 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>石岡區</t>
+          <t>大甲區</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>石岡市區</t>
+          <t>大甲市區</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -6329,12 +6329,12 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>石岡區</t>
+          <t>大甲區</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>中山路</t>
+          <t>大甲媽祖</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -6346,12 +6346,12 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>石岡區</t>
+          <t>大甲區</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>食水嵙</t>
+          <t>中山路</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -6363,12 +6363,12 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>石岡區</t>
+          <t>大甲區</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>三叉坑</t>
+          <t>蔣公路</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -6380,12 +6380,12 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>和平區</t>
+          <t>外埔區</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>梨山</t>
+          <t>外埔市區</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -6397,12 +6397,12 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>和平區</t>
+          <t>外埔區</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>武陵農場</t>
+          <t>中山路</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -6414,12 +6414,12 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>和平區</t>
+          <t>外埔區</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>谷關溫泉</t>
+          <t>大甲溪</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -6431,15 +6431,83 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>和平區</t>
+          <t>外埔區</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>環山部落</t>
+          <t>水美溫泉</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>大安區</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>大安市區</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>大安區</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>大安漁港</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>大安區</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>中山路</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>大安區</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>海岸線</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
         <is>
           <t>商圈</t>
         </is>

</xml_diff>